<commit_message>
publish_windowed: rebuild window @ 20260922-223249
</commit_message>
<xml_diff>
--- a/weeks/2026-09-17/巡查表.xlsx
+++ b/weeks/2026-09-17/巡查表.xlsx
@@ -7307,7 +7307,7 @@
       </c>
       <c r="N63" t="inlineStr">
         <is>
-          <t>1.5: 至少设置一处有害垃圾收集容器。（5分） (5)</t>
+          <t>1.5: 至少设置一处有害垃圾收集容器。（5分） (-5)</t>
         </is>
       </c>
       <c r="O63" s="4" t="inlineStr">
@@ -11060,7 +11060,7 @@
       </c>
       <c r="O96" s="4" t="inlineStr">
         <is>
-          <t>查看证据(8项/10张)</t>
+          <t>查看证据(8项/19张)</t>
         </is>
       </c>
       <c r="P96" t="n">
@@ -19241,7 +19241,7 @@
       </c>
       <c r="O170" s="4" t="inlineStr">
         <is>
-          <t>查看证据(4项/3张)</t>
+          <t>查看证据(4项/4张)</t>
         </is>
       </c>
       <c r="P170" t="n">
@@ -21518,7 +21518,7 @@
       </c>
       <c r="N190" t="inlineStr">
         <is>
-          <t>1.5: 至少设置一处有害垃圾收集容器。（5分） (5)
+          <t>1.5: 至少设置一处有害垃圾收集容器。（5分） (-5)
 1.6: 各类收集容器的分类标志完整、正确、清晰。 （12分） (-3)</t>
         </is>
       </c>
@@ -21875,7 +21875,7 @@
       </c>
       <c r="O193" s="4" t="inlineStr">
         <is>
-          <t>查看证据(3项/4张)</t>
+          <t>查看证据(3项/7张)</t>
         </is>
       </c>
       <c r="P193" t="n">
@@ -28370,7 +28370,7 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="F157" s="6" t="inlineStr">
@@ -41579,7 +41579,7 @@
       </c>
       <c r="E514" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="F514" s="6" t="inlineStr">

</xml_diff>